<commit_message>
Actualizar proyecto de acuerdo a la versión de Acme-Framework 26.2.0
</commit_message>
<xml_diff>
--- a/reports/Deliverable D01 (Level C)/Group/Planning-Template.xlsx
+++ b/reports/Deliverable D01 (Level C)/Group/Planning-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javier\Downloads\Workspace-26\Projects\Acme-Starters-C\reports\Deliverable D01 (Level C)\Group\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63FE3EB7-2DB7-4016-9261-F5AA9A177B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1120C43-8129-4DDD-94CE-1E864276BC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
   </bookViews>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E7" s="36">
         <f>SUM(O12:O112)</f>
-        <v>378.33333333333331</v>
+        <v>395</v>
       </c>
       <c r="J7" s="37"/>
     </row>
@@ -2710,22 +2710,26 @@
       <c r="I28" s="46">
         <v>46066.006944444445</v>
       </c>
-      <c r="J28" s="46"/>
+      <c r="J28" s="46">
+        <v>46066.034722222219</v>
+      </c>
       <c r="K28" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>Ongoing</v>
       </c>
       <c r="L28" s="47">
         <v>0.33333333333333331</v>
       </c>
-      <c r="M28" s="47"/>
+      <c r="M28" s="47">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="N28" s="45">
         <f>IF(ISBLANK(L28), "", L28*VLOOKUP($F28,Internal!$B$26:$C$32,2,FALSE))</f>
         <v>8.3333333333333321</v>
       </c>
-      <c r="O28" s="45" t="str">
+      <c r="O28" s="45">
         <f>IF(ISBLANK(M28), "", M28*VLOOKUP($F28,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
+        <v>16.666666666666664</v>
       </c>
       <c r="P28" s="44" t="s">
         <v>110</v>

</xml_diff>

<commit_message>
Implementar requisito S1/1 sin validaciones personalizadas ni adicionales
</commit_message>
<xml_diff>
--- a/reports/Deliverable D01 (Level C)/Group/Planning-Template.xlsx
+++ b/reports/Deliverable D01 (Level C)/Group/Planning-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Javier\Downloads\Workspace-26\Projects\Acme-Starters-C\reports\Deliverable D01 (Level C)\Group\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1120C43-8129-4DDD-94CE-1E864276BC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104EF387-DBB9-48A9-9AE3-297D933BB532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{683E09B8-1D94-4905-B116-9D998A46AAA3}"/>
   </bookViews>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E7" s="36">
         <f>SUM(O12:O112)</f>
-        <v>395</v>
+        <v>470</v>
       </c>
       <c r="J7" s="37"/>
     </row>
@@ -2391,22 +2391,26 @@
       <c r="I21" s="46">
         <v>46065.708333333336</v>
       </c>
-      <c r="J21" s="46"/>
+      <c r="J21" s="46">
+        <v>46067.578472222223</v>
+      </c>
       <c r="K21" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>Completed</v>
       </c>
       <c r="L21" s="47">
         <v>3</v>
       </c>
-      <c r="M21" s="47"/>
+      <c r="M21" s="47">
+        <v>3</v>
+      </c>
       <c r="N21" s="45">
         <f>IF(ISBLANK(L21), "", L21*VLOOKUP($F21,Internal!$B$26:$C$32,2,FALSE))</f>
         <v>75</v>
       </c>
-      <c r="O21" s="45" t="str">
+      <c r="O21" s="45">
         <f>IF(ISBLANK(M21), "", M21*VLOOKUP($F21,Internal!$B$26:$C$32,2,FALSE))</f>
-        <v/>
+        <v>75</v>
       </c>
       <c r="P21" s="44" t="s">
         <v>104</v>
@@ -2715,7 +2719,7 @@
       </c>
       <c r="K28" s="45" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>Ongoing</v>
+        <v>Completed</v>
       </c>
       <c r="L28" s="47">
         <v>0.33333333333333331</v>

</xml_diff>